<commit_message>
fixed reference number script
</commit_message>
<xml_diff>
--- a/product family/MX123/MX123 49 CKT WDC (216744)/Reference Numbers.xlsx
+++ b/product family/MX123/MX123 49 CKT WDC (216744)/Reference Numbers.xlsx
@@ -533,7 +533,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>DRESS COVER BLACK-34575-0005</t>
+          <t>DRESS COVER-34575-0005</t>
         </is>
       </c>
     </row>
@@ -571,7 +571,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>DRESS COVER BLACK-34575-0005</t>
+          <t>DRESS COVER-34575-0005</t>
         </is>
       </c>
     </row>
@@ -609,7 +609,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>DRESS COVER BLACK-34575-0005</t>
+          <t>DRESS COVER-34575-0005</t>
         </is>
       </c>
     </row>
@@ -647,7 +647,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>DRESS COVER BLACK-34575-0005</t>
+          <t>DRESS COVER-34575-0005</t>
         </is>
       </c>
     </row>
@@ -685,7 +685,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>DRESS COVER BLACK-34575-0005</t>
+          <t>DRESS COVER-34575-0005</t>
         </is>
       </c>
     </row>
@@ -723,7 +723,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>DRESS COVER BLACK-34575-0005</t>
+          <t>DRESS COVER-34575-0005</t>
         </is>
       </c>
     </row>
@@ -761,7 +761,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>DRESS COVER BLACK-34575-0005</t>
+          <t>DRESS COVER-34575-0005</t>
         </is>
       </c>
     </row>
@@ -799,7 +799,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>DRESS COVER BLACK-34575-0005</t>
+          <t>DRESS COVER-34575-0005</t>
         </is>
       </c>
     </row>

</xml_diff>